<commit_message>
new figures for rgaphical abstract
</commit_message>
<xml_diff>
--- a/data/data_extraction/decisions_for_exclusion.xlsx
+++ b/data/data_extraction/decisions_for_exclusion.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\j_stee03\Sciebo\Review take off\data\data_extraction\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\j_stee03\Uni\takeoff\data\data_extraction\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72BC3A5F-983E-41C5-86BA-8050A43DDB73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C853451-3216-458D-BEE8-1FC38A78765E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38520" yWindow="30" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="include" sheetId="1" r:id="rId1"/>

</xml_diff>